<commit_message>
En Simulació venda, deso l'any renda al registre Windows, per que persisteixi el valor en la següent arrancada.
</commit_message>
<xml_diff>
--- a/Docs/Arcelor-Perdues desde2018.xlsx
+++ b/Docs/Arcelor-Perdues desde2018.xlsx
@@ -169,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -199,6 +199,9 @@
     <xf numFmtId="8" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -578,7 +581,7 @@
     <col min="17" max="17" width="11.453125" customWidth="1"/>
     <col min="18" max="18" width="10" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="9.90625" customWidth="1"/>
-    <col min="20" max="20" width="8.7265625" customWidth="1"/>
+    <col min="20" max="20" width="9.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15" thickBot="1">
@@ -1101,30 +1104,30 @@
         <f>SUM(O14:P14)</f>
         <v>2499.7899999999936</v>
       </c>
-      <c r="R14" s="30">
+      <c r="R14" s="31">
         <f>SUM(Q11:Q14)</f>
         <v>1259.9499999999898</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="15" thickBot="1">
-      <c r="A15" s="27"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28"/>
-      <c r="K15" s="28"/>
-      <c r="L15" s="28"/>
-      <c r="M15" s="28"/>
-      <c r="N15" s="28"/>
-      <c r="O15" s="28"/>
-      <c r="P15" s="28"/>
-      <c r="Q15" s="28"/>
-      <c r="R15" s="26"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
+      <c r="I15" s="29"/>
+      <c r="J15" s="29"/>
+      <c r="K15" s="29"/>
+      <c r="L15" s="29"/>
+      <c r="M15" s="29"/>
+      <c r="N15" s="29"/>
+      <c r="O15" s="29"/>
+      <c r="P15" s="29"/>
+      <c r="Q15" s="29"/>
+      <c r="R15" s="27"/>
     </row>
     <row r="16" spans="1:18">
       <c r="A16" s="6">
@@ -1282,6 +1285,9 @@
       <c r="P19" s="13"/>
       <c r="Q19" s="13"/>
       <c r="R19" s="17"/>
+      <c r="S19" s="1">
+        <v>3985.29</v>
+      </c>
     </row>
     <row r="20" spans="1:20">
       <c r="A20" s="12">
@@ -1323,6 +1329,9 @@
       <c r="P20" s="13"/>
       <c r="Q20" s="13"/>
       <c r="R20" s="17"/>
+      <c r="S20" s="1">
+        <v>-3998.58</v>
+      </c>
     </row>
     <row r="21" spans="1:20" ht="15" thickBot="1">
       <c r="A21" s="18"/>
@@ -1360,6 +1369,10 @@
         <f>SUM(Q18:Q21)</f>
         <v>-7.2705499999992753</v>
       </c>
+      <c r="S21" s="1">
+        <f>SUM(S19:S20)</f>
+        <v>-13.289999999999964</v>
+      </c>
     </row>
     <row r="22" spans="1:20">
       <c r="A22" s="6">
@@ -1555,6 +1568,9 @@
         <f>SUM(Q25:Q26)</f>
         <v>-9095.8608785714277</v>
       </c>
+      <c r="S26" s="1">
+        <v>-9089.81</v>
+      </c>
     </row>
     <row r="27" spans="1:20">
       <c r="A27" s="6">
@@ -1787,6 +1803,9 @@
         <v>629.33297124600631</v>
       </c>
       <c r="R32" s="17"/>
+      <c r="S32" s="1">
+        <v>1079.8399999999999</v>
+      </c>
     </row>
     <row r="33" spans="1:20">
       <c r="A33" s="12"/>
@@ -1821,6 +1840,9 @@
         <v>112.58830670926545</v>
       </c>
       <c r="R33" s="17"/>
+      <c r="S33" s="1">
+        <v>-577.44000000000005</v>
+      </c>
     </row>
     <row r="34" spans="1:20" ht="15" thickBot="1">
       <c r="A34" s="18"/>
@@ -1858,9 +1880,14 @@
         <f>SUM(Q31:Q34)</f>
         <v>495.56506493506549</v>
       </c>
+      <c r="S34" s="1">
+        <f>SUM(S32:S33)</f>
+        <v>502.39999999999986</v>
+      </c>
     </row>
     <row r="35" spans="1:20">
       <c r="O35" s="3"/>
+      <c r="Q35" s="1"/>
       <c r="R35" s="24">
         <f>SUM(R16:R34)</f>
         <v>-8607.5663636363606</v>
@@ -1907,6 +1934,12 @@
       </c>
       <c r="N36" s="3"/>
       <c r="O36" s="1"/>
+      <c r="Q36" s="25">
+        <v>-7.27</v>
+      </c>
+      <c r="R36" s="24">
+        <v>2664.31</v>
+      </c>
     </row>
     <row r="37" spans="1:20">
       <c r="A37">
@@ -1940,6 +1973,13 @@
         <f>K36+D37</f>
         <v>1467</v>
       </c>
+      <c r="Q37" s="25">
+        <v>-9095.86</v>
+      </c>
+      <c r="R37" s="1">
+        <f>SUM(R35:R36)</f>
+        <v>-5943.2563636363611</v>
+      </c>
     </row>
     <row r="38" spans="1:20">
       <c r="A38">
@@ -1973,6 +2013,9 @@
         <f>K37+D38</f>
         <v>1900</v>
       </c>
+      <c r="Q38" s="25">
+        <v>3125.41</v>
+      </c>
     </row>
     <row r="39" spans="1:20">
       <c r="A39">
@@ -2006,16 +2049,19 @@
         <f>K38-D39</f>
         <v>1900</v>
       </c>
-      <c r="Q39" s="1"/>
+      <c r="Q39" s="1">
+        <f>SUM(Q36:Q38)</f>
+        <v>-5977.7200000000012</v>
+      </c>
       <c r="R39" s="24"/>
     </row>
     <row r="44" spans="1:20">
-      <c r="F44" s="25">
+      <c r="F44" s="26">
         <v>-3998.58</v>
       </c>
     </row>
     <row r="45" spans="1:20">
-      <c r="F45" s="25">
+      <c r="F45" s="26">
         <v>3985.29</v>
       </c>
     </row>
@@ -2023,19 +2069,31 @@
       <c r="E46">
         <v>2018</v>
       </c>
-      <c r="F46" s="25">
+      <c r="F46" s="26">
         <f>SUM(F44:F45)</f>
         <v>-13.289999999999964</v>
       </c>
+      <c r="R46">
+        <v>2021</v>
+      </c>
     </row>
     <row r="47" spans="1:20">
       <c r="F47" s="1"/>
+      <c r="R47">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20">
+      <c r="R48">
+        <f>+R46-R47</f>
+        <v>2017</v>
+      </c>
     </row>
     <row r="49" spans="5:6">
       <c r="E49">
         <v>2019</v>
       </c>
-      <c r="F49" s="25">
+      <c r="F49" s="26">
         <v>-9089.81</v>
       </c>
     </row>

</xml_diff>